<commit_message>
Changes done on UAT
</commit_message>
<xml_diff>
--- a/Data/Modifier_log_Template.xlsx
+++ b/Data/Modifier_log_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKR7550\Documents\RE_CFCAutomation\RE_CFCAutomation\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKR7550\Documents\UiPath\RPA_CFC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C846D93-5B47-44E1-892C-AE5ED1DE90CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{911FF826-75D1-448A-A232-59A4C2B30550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{3203513D-5511-4B48-8E59-55BB4D7708A1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Action</t>
   </si>
@@ -50,13 +50,7 @@
     <t>MG_ID</t>
   </si>
   <si>
-    <t>Items Addedd</t>
-  </si>
-  <si>
-    <t>Items Deleted</t>
-  </si>
-  <si>
-    <t>Exception_Details</t>
+    <t>Exception Details</t>
   </si>
 </sst>
 </file>
@@ -459,19 +453,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10DE1B90-BA82-4B98-9093-0B8DADE7BBCD}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="17" style="2" customWidth="1"/>
     <col min="3" max="3" width="28.42578125" style="2" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="32" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="28.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="28.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -487,12 +479,6 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>